<commit_message>
add Python load script and SQL views - database layer complete
</commit_message>
<xml_diff>
--- a/cost-plans/Data-Centre-Shell-and-Core.xlsx
+++ b/cost-plans/Data-Centre-Shell-and-Core.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\qs\project-cost-control\cost-plans\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECDD3EBE-0CF7-4683-B576-5B198ECCF581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3F81D4D-71F1-4908-BEB5-581A52B9ABB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14092" activeTab="1" xr2:uid="{0C8C6BE1-598D-4333-9AA5-A074653745B1}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14092" activeTab="2" xr2:uid="{0C8C6BE1-598D-4333-9AA5-A074653745B1}"/>
   </bookViews>
   <sheets>
     <sheet name="Cost Plan" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="78">
   <si>
     <t>Project Name</t>
   </si>
@@ -184,18 +184,6 @@
     <t>EAC</t>
   </si>
   <si>
-    <t>Urban Highway Improvement Scheme</t>
-  </si>
-  <si>
-    <t>Transport for Greater Manchester</t>
-  </si>
-  <si>
-    <t>NEC4 Engineering and Construction Contract</t>
-  </si>
-  <si>
-    <t>Urban Highway Improvement Scheme — Elemental Cost Plan</t>
-  </si>
-  <si>
     <t>4.1</t>
   </si>
   <si>
@@ -269,6 +257,24 @@
   </si>
   <si>
     <t>Meridian Cost Consultants | Reporting Period: March 2026</t>
+  </si>
+  <si>
+    <t>Sector</t>
+  </si>
+  <si>
+    <t>Commercial</t>
+  </si>
+  <si>
+    <t>Data Centre Shell &amp; Core— Elemental Cost Plan</t>
+  </si>
+  <si>
+    <t>Data Centre Shell &amp; Core</t>
+  </si>
+  <si>
+    <t>TechNorth Digital Infrastructure Ltd</t>
+  </si>
+  <si>
+    <t>JCT Design and Build 2016</t>
   </si>
 </sst>
 </file>
@@ -520,21 +526,13 @@
   <dxfs count="5">
     <dxf>
       <font>
+        <b/>
+        <i val="0"/>
         <color theme="0"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -552,13 +550,21 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
         <color theme="0"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1970,7 +1976,7 @@
   <sheetData>
     <row r="1" spans="1:10" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="46" t="s">
-        <v>50</v>
+        <v>74</v>
       </c>
       <c r="B1" s="46"/>
       <c r="C1" s="46"/>
@@ -1985,7 +1991,7 @@
     <row r="2" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="47" t="str">
         <f ca="1">"Meridian Cost Consultants | Report Date: "&amp;TEXT(TODAY(),"DD MMMM YYYY")</f>
-        <v>Meridian Cost Consultants | Report Date: 15 May 2026</v>
+        <v>Meridian Cost Consultants | Report Date: 16 May 2026</v>
       </c>
       <c r="B2" s="47"/>
       <c r="C2" s="47"/>
@@ -2034,14 +2040,14 @@
         <v>20</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C5" s="28">
         <f>SUM(C6:C7)</f>
         <v>1320000</v>
       </c>
       <c r="D5" s="28">
-        <f t="shared" ref="D5:I20" si="0">SUM(D6:D7)</f>
+        <f t="shared" ref="D5:I5" si="0">SUM(D6:D7)</f>
         <v>0</v>
       </c>
       <c r="E5" s="28">
@@ -2074,7 +2080,7 @@
         <v>21</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C6" s="29">
         <v>880000</v>
@@ -2106,7 +2112,7 @@
         <v>22</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C7" s="30">
         <v>440000</v>
@@ -2138,7 +2144,7 @@
         <v>23</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C8" s="28">
         <f>SUM(C9:C11)</f>
@@ -2178,7 +2184,7 @@
         <v>24</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C9" s="29">
         <v>1320000</v>
@@ -2210,7 +2216,7 @@
         <v>25</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C10" s="30">
         <v>660000</v>
@@ -2242,7 +2248,7 @@
         <v>26</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C11" s="29">
         <v>880000</v>
@@ -2274,7 +2280,7 @@
         <v>27</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C12" s="28">
         <f>SUM(C13:C14)</f>
@@ -2314,7 +2320,7 @@
         <v>28</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C13" s="29">
         <v>440000</v>
@@ -2346,7 +2352,7 @@
         <v>29</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C14" s="30">
         <v>660000</v>
@@ -2378,7 +2384,7 @@
         <v>30</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C15" s="28">
         <f>SUM(C16:C19)</f>
@@ -2415,10 +2421,10 @@
     </row>
     <row r="16" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A16" s="9" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="C16" s="29">
         <v>4840000</v>
@@ -2449,10 +2455,10 @@
     </row>
     <row r="17" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A17" s="10" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C17" s="30">
         <v>3520000</v>
@@ -2481,10 +2487,10 @@
     </row>
     <row r="18" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A18" s="9" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C18" s="29">
         <v>1760000</v>
@@ -2515,10 +2521,10 @@
     </row>
     <row r="19" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A19" s="9" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C19" s="29">
         <v>1100000</v>
@@ -2550,7 +2556,7 @@
         <v>31</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C20" s="28">
         <f>SUM(C21:C22)</f>
@@ -2590,7 +2596,7 @@
         <v>32</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C21" s="29">
         <v>660000</v>
@@ -2622,7 +2628,7 @@
         <v>33</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C22" s="30">
         <v>440000</v>
@@ -2654,7 +2660,7 @@
         <v>34</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C23" s="28">
         <v>880000</v>
@@ -2790,13 +2796,13 @@
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <conditionalFormatting sqref="I5:I26">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="4" priority="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>AND(I5&lt;0, I5&gt;=-E5*0.02)</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="3" operator="lessThan">
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2823,7 +2829,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="46" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B1" s="46"/>
       <c r="C1" s="46"/>
@@ -2834,7 +2840,7 @@
     </row>
     <row r="2" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="47" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B2" s="47"/>
       <c r="C2" s="47"/>
@@ -2936,10 +2942,10 @@
     <mergeCell ref="A2:G2"/>
   </mergeCells>
   <conditionalFormatting sqref="D5:D23">
-    <cfRule type="expression" dxfId="4" priority="1">
+    <cfRule type="expression" dxfId="1" priority="1">
       <formula>D5&gt;0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="2">
+    <cfRule type="expression" dxfId="0" priority="2">
       <formula>D5&lt;0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2950,7 +2956,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2FB73FC-2423-441D-B32D-DF5AF30B74F5}">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="25.69140625" bestFit="1" customWidth="1"/>
@@ -2962,7 +2968,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="22" t="s">
-        <v>47</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.4">
@@ -2970,7 +2976,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>48</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.4">
@@ -2978,7 +2984,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>49</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.4">
@@ -2986,7 +2992,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="24">
-        <v>32000000</v>
+        <v>22000000</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.4">
@@ -2994,7 +3000,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="25">
-        <v>45170</v>
+        <v>46054</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.4">
@@ -3002,7 +3008,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="26">
-        <v>46081</v>
+        <v>46783</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.4">
@@ -3028,6 +3034,14 @@
       <c r="B9" s="27">
         <f>'Cost Plan'!J26</f>
         <v>0.1079231845351647</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A10" s="21" t="s">
+        <v>72</v>
+      </c>
+      <c r="B10" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>